<commit_message>
Read Me Updated, Notebooks Updates
</commit_message>
<xml_diff>
--- a/notebooks/products.xlsx
+++ b/notebooks/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -433,6 +433,186 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>8719587102916</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2025-07-02 19:42:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>9718787102916</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2025-07-02 19:42:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>9005800329604</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2025-07-02 19:44:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0084000005807</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2025-07-02 19:45:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>9106224329604</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2025-07-02 19:45:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>8001100329604</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2025-07-02 20:15:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>9005200389604</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2025-07-02 20:15:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1046283329604</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2025-07-02 20:15:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>9007200329604</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2025-07-02 20:16:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>3045000329604</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2025-07-02 20:16:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>5005828329604</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2025-07-02 20:52:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0941220329604</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2025-07-02 20:54:33</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>